<commit_message>
feat: add project-site kitchen equipment tracking
</commit_message>
<xml_diff>
--- a/docs/data-import-templates/company_erp_mvp_import_templates.xlsx
+++ b/docs/data-import-templates/company_erp_mvp_import_templates.xlsx
@@ -393,7 +393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,35 +449,45 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>合同形态*</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>合同标的分类*</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>签订日期</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>开始日期</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>结束日期</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>合同金额</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>状态*</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>附件路径</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -516,33 +526,43 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>框架合同</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>厨房设备</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2027-05-31</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>120000</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>履行中</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>attachments/contracts/HT202605001.pdf</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>示例行</t>
         </is>
@@ -616,7 +636,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -814,32 +833,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -882,7 +875,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -1040,32 +1032,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -1108,7 +1074,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -1233,32 +1198,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -1284,7 +1223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1892,6 +1831,134 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>外部经理账号不绑定员工，不作为合同相对方。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>合同台账</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>合同方向</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>字典</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>采购合同</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>只允许采购合同、甲方服务合同、外包合同、其他；框架不再作为合同方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>合同台账</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>合同形态</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>字典</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>框架合同</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>只允许一次性合同、固定期限合同、框架合同、工程/建设合同。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>合同台账</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>合同标的分类</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>字典</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>厨房设备</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>只允许食材、餐具用品、厨房设备、广告标识/广告制作、装修/改造、土建/厂房/土地建设、电梯、团餐/食堂运营服务、分包/外包服务、其他。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>合同台账</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>字典</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>只允许草稿、履行中、已完成、已终止、已取消；已完成由人工确认。</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2127,6 +2194,74 @@
       <c r="C13" t="inlineStr">
         <is>
           <t>项目点外部项目经理账号状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>合同方向</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>采购合同 / 甲方服务合同 / 外包合同 / 其他</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>合同方向回答和谁签、业务关系是什么；框架不作为方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>合同形态</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>一次性合同 / 固定期限合同 / 框架合同 / 工程/建设合同</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>合同形态回答一次性、固定期限、框架还是工程建设。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>合同标的分类</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>食材 / 餐具用品 / 厨房设备 / 广告标识/广告制作 / 装修/改造 / 土建/厂房/土地建设 / 电梯 / 团餐/食堂运营服务 / 分包/外包服务 / 其他</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>合同标的分类回答买、做或服务的内容。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>合同状态</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>草稿 / 履行中 / 已完成 / 已终止 / 已取消</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>业务状态人工维护；到期状态由结束日期派生展示。</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2171,7 +2306,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2299,7 +2433,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2421,7 +2554,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2551,32 +2683,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -2626,7 +2732,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2739,32 +2844,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -2814,7 +2893,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2937,32 +3015,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3012,7 +3064,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3203,32 +3254,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3271,7 +3296,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3371,32 +3395,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3449,7 +3447,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3599,32 +3596,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3674,7 +3645,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3775,32 +3745,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3850,7 +3794,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3993,32 +3936,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add project-site kitchen equipment tracking (#35)
</commit_message>
<xml_diff>
--- a/docs/data-import-templates/company_erp_mvp_import_templates.xlsx
+++ b/docs/data-import-templates/company_erp_mvp_import_templates.xlsx
@@ -393,7 +393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,35 +449,45 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>合同形态*</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>合同标的分类*</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>签订日期</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>开始日期</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>结束日期</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>合同金额</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>状态*</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>附件路径</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -516,33 +526,43 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>框架合同</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>厨房设备</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2027-05-31</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>120000</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>履行中</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>attachments/contracts/HT202605001.pdf</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>示例行</t>
         </is>
@@ -616,7 +636,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -814,32 +833,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -882,7 +875,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -1040,32 +1032,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -1108,7 +1074,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -1233,32 +1198,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -1284,7 +1223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1892,6 +1831,134 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>外部经理账号不绑定员工，不作为合同相对方。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>合同台账</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>合同方向</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>字典</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>采购合同</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>只允许采购合同、甲方服务合同、外包合同、其他；框架不再作为合同方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>合同台账</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>合同形态</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>字典</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>框架合同</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>只允许一次性合同、固定期限合同、框架合同、工程/建设合同。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>合同台账</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>合同标的分类</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>字典</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>厨房设备</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>只允许食材、餐具用品、厨房设备、广告标识/广告制作、装修/改造、土建/厂房/土地建设、电梯、团餐/食堂运营服务、分包/外包服务、其他。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>合同台账</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>字典</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>只允许草稿、履行中、已完成、已终止、已取消；已完成由人工确认。</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2127,6 +2194,74 @@
       <c r="C13" t="inlineStr">
         <is>
           <t>项目点外部项目经理账号状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>合同方向</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>采购合同 / 甲方服务合同 / 外包合同 / 其他</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>合同方向回答和谁签、业务关系是什么；框架不作为方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>合同形态</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>一次性合同 / 固定期限合同 / 框架合同 / 工程/建设合同</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>合同形态回答一次性、固定期限、框架还是工程建设。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>合同标的分类</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>食材 / 餐具用品 / 厨房设备 / 广告标识/广告制作 / 装修/改造 / 土建/厂房/土地建设 / 电梯 / 团餐/食堂运营服务 / 分包/外包服务 / 其他</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>合同标的分类回答买、做或服务的内容。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>合同状态</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>草稿 / 履行中 / 已完成 / 已终止 / 已取消</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>业务状态人工维护；到期状态由结束日期派生展示。</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2171,7 +2306,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2299,7 +2433,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2421,7 +2554,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2551,32 +2683,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -2626,7 +2732,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2739,32 +2844,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -2814,7 +2893,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2937,32 +3015,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3012,7 +3064,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3203,32 +3254,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3271,7 +3296,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3371,32 +3395,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3449,7 +3447,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3599,32 +3596,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3674,7 +3645,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3775,32 +3745,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -3850,7 +3794,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3993,32 +3936,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>

</xml_diff>